<commit_message>
feat(address): stabilize address form and add test retry logic - Configured automatic retry (retry: 2) in cucumber.conf.js and retry buffer wait in hooks.js. - Added comprehensive GETTING_STARTED.md with framework architecture.
</commit_message>
<xml_diff>
--- a/features/testdata/contractor_employee-combo.xlsx
+++ b/features/testdata/contractor_employee-combo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CLMS-Automation\testing-framework-playwright--simplecode\features\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BBCC595-075F-4B01-9037-027335155804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE00AE7-A6A3-4D61-A1D6-A550B4592F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContratorEmployee" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="186">
   <si>
     <t>EmployeeCode</t>
   </si>
@@ -483,9 +483,6 @@
     <t>IsAutoShiftApplicable</t>
   </si>
   <si>
-    <t>Sharma</t>
-  </si>
-  <si>
     <t>K</t>
   </si>
   <si>
@@ -546,30 +543,15 @@
     <t>Semi-Skilled</t>
   </si>
   <si>
-    <t>1001</t>
-  </si>
-  <si>
-    <t>1004</t>
-  </si>
-  <si>
     <t>OT Applicable</t>
   </si>
   <si>
     <t>Hinduism</t>
   </si>
   <si>
-    <t xml:space="preserve">Isha </t>
-  </si>
-  <si>
-    <t>Rana</t>
-  </si>
-  <si>
     <t>A+</t>
   </si>
   <si>
-    <t>1002</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
@@ -577,6 +559,30 @@
   </si>
   <si>
     <t>P</t>
+  </si>
+  <si>
+    <t>Kamat</t>
+  </si>
+  <si>
+    <t>Hajare</t>
+  </si>
+  <si>
+    <t>Shantanu</t>
+  </si>
+  <si>
+    <t>Raghawan</t>
+  </si>
+  <si>
+    <t>6456111111BBB9999</t>
+  </si>
+  <si>
+    <t>Bhophalekar</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Gokul</t>
   </si>
 </sst>
 </file>
@@ -619,11 +625,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -654,7 +661,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ContratorEmployee" displayName="ContratorEmployee" ref="A1:EV4" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ContratorEmployee" displayName="ContratorEmployee" ref="A1:EV5" totalsRowShown="0">
   <tableColumns count="152">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="EmployeeCode"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="FirstName"/>
@@ -1098,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EV4"/>
+  <dimension ref="A1:EV5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" customWidth="1"/>
@@ -1699,37 +1706,34 @@
     </row>
     <row r="2" spans="1:152" ht="15.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>66324760000</v>
+        <v>7660001</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>180</v>
       </c>
       <c r="D2" t="s">
-        <v>153</v>
+        <v>181</v>
       </c>
       <c r="G2" s="1">
         <v>32697</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>154</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>174</v>
+      </c>
+      <c r="K2" t="s">
         <v>155</v>
       </c>
-      <c r="J2" t="s">
-        <v>179</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>156</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>157</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>158</v>
-      </c>
-      <c r="O2" t="s">
-        <v>159</v>
       </c>
       <c r="P2" s="1">
         <v>46044</v>
@@ -1738,189 +1742,186 @@
         <v>199</v>
       </c>
       <c r="R2" t="s">
+        <v>159</v>
+      </c>
+      <c r="T2" t="s">
         <v>160</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>161</v>
       </c>
-      <c r="U2" t="s">
+      <c r="AA2" s="4">
+        <v>906740241455</v>
+      </c>
+      <c r="AI2" t="s">
         <v>162</v>
       </c>
-      <c r="AA2">
-        <v>9067452489</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>163</v>
-      </c>
       <c r="AJ2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AK2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AL2">
         <v>0</v>
       </c>
       <c r="AM2" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN2" t="s">
         <v>163</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AO2" t="s">
+        <v>162</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>163</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>162</v>
+      </c>
+      <c r="AV2" t="s">
         <v>164</v>
       </c>
-      <c r="AO2" t="s">
-        <v>163</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>164</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>160</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>160</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>163</v>
-      </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>165</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AX2" t="s">
         <v>166</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AY2" t="s">
         <v>167</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="BA2" t="s">
         <v>168</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BB2" t="s">
+        <v>175</v>
+      </c>
+      <c r="BC2" t="s">
         <v>169</v>
       </c>
-      <c r="BB2" t="s">
-        <v>181</v>
-      </c>
-      <c r="BC2" t="s">
+      <c r="BD2" t="s">
         <v>170</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BE2" t="s">
         <v>171</v>
       </c>
-      <c r="BE2" t="s">
-        <v>172</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>173</v>
+      <c r="BF2">
+        <v>1001</v>
       </c>
       <c r="BG2" s="1">
         <v>46228</v>
       </c>
-      <c r="BH2" t="s">
-        <v>174</v>
+      <c r="BH2">
+        <v>1004</v>
       </c>
       <c r="BQ2" s="3">
-        <v>965236585254</v>
+        <v>300181818</v>
       </c>
       <c r="CY2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DA2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DC2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DE2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DG2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DI2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DS2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DT2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DU2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DV2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="DW2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="DX2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="DY2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="DZ2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="EA2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="EB2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="EC2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="ED2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="EF2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="EH2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="EJ2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="EK2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="EL2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="EU2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="EV2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:152" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>32476</v>
-      </c>
       <c r="B3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G3" s="1">
         <v>32831</v>
       </c>
       <c r="H3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J3" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="M3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="P3" s="1">
         <v>46056</v>
@@ -1929,49 +1930,46 @@
         <v>67</v>
       </c>
       <c r="T3" t="s">
+        <v>160</v>
+      </c>
+      <c r="U3" t="s">
         <v>161</v>
       </c>
-      <c r="U3" t="s">
+      <c r="AA3" s="4">
+        <v>600010100997</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>159</v>
+      </c>
+      <c r="AT3" t="s">
         <v>162</v>
       </c>
-      <c r="AA3">
-        <v>5017152411</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>160</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>163</v>
-      </c>
       <c r="AV3" t="s">
+        <v>164</v>
+      </c>
+      <c r="AW3" t="s">
         <v>165</v>
       </c>
-      <c r="AW3" t="s">
+      <c r="AX3" t="s">
         <v>166</v>
       </c>
-      <c r="AX3" t="s">
+      <c r="AY3" t="s">
         <v>167</v>
       </c>
-      <c r="AY3" t="s">
+      <c r="BA3" t="s">
         <v>168</v>
       </c>
-      <c r="BA3" t="s">
+      <c r="BB3" t="s">
+        <v>175</v>
+      </c>
+      <c r="BC3" t="s">
         <v>169</v>
       </c>
-      <c r="BB3" t="s">
-        <v>181</v>
-      </c>
-      <c r="BC3" t="s">
+      <c r="BD3" t="s">
         <v>170</v>
       </c>
-      <c r="BD3" t="s">
+      <c r="BE3" t="s">
         <v>171</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>172</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>180</v>
       </c>
       <c r="BG3" s="2"/>
       <c r="BH3">
@@ -1983,15 +1981,153 @@
         <v>6736632</v>
       </c>
       <c r="B4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4" t="s">
+        <v>152</v>
+      </c>
+      <c r="H4" t="s">
+        <v>177</v>
+      </c>
+      <c r="T4" t="s">
+        <v>160</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>164</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>165</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>166</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>167</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>168</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>175</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>169</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>170</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>171</v>
+      </c>
+      <c r="BG4" s="2"/>
+      <c r="BH4">
+        <v>1004</v>
+      </c>
+      <c r="BQ4" t="s">
         <v>182</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:152" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>500901</v>
+      </c>
+      <c r="B5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G5" s="1">
+        <v>34657</v>
+      </c>
+      <c r="H5" t="s">
         <v>153</v>
       </c>
-      <c r="H4" t="s">
-        <v>183</v>
-      </c>
-      <c r="BG4" s="2"/>
+      <c r="J5" t="s">
+        <v>174</v>
+      </c>
+      <c r="K5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>156</v>
+      </c>
+      <c r="N5" t="s">
+        <v>184</v>
+      </c>
+      <c r="O5" t="s">
+        <v>158</v>
+      </c>
+      <c r="P5" s="1">
+        <v>46068</v>
+      </c>
+      <c r="Q5">
+        <v>77</v>
+      </c>
+      <c r="T5" t="s">
+        <v>160</v>
+      </c>
+      <c r="U5" t="s">
+        <v>161</v>
+      </c>
+      <c r="AA5" s="4">
+        <v>903343243333</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>159</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>162</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>163</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>159</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>159</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>162</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>164</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>165</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>166</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>167</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>168</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>175</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>169</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>170</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>171</v>
+      </c>
+      <c r="BF5">
+        <v>1001</v>
+      </c>
+      <c r="BG5" s="2"/>
+      <c r="BH5">
+        <v>1004</v>
+      </c>
+      <c r="BQ5" s="3">
+        <v>520200133800</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>